<commit_message>
Other income and changes updated
</commit_message>
<xml_diff>
--- a/MASTER DRAFT .xlsx
+++ b/MASTER DRAFT .xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{016C980B-588C-47EA-B7F3-1DE75E065E2F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{016C980B-588C-47EA-B7F3-1DE75E065E2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QUOTE FORMATE" sheetId="2" r:id="rId1"/>
@@ -22,6 +22,17 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -1565,12 +1576,12 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="25" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1592,53 +1603,29 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1683,6 +1670,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="18" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="19" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1753,7 +1746,55 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="18" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="16" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="16" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1776,56 +1817,14 @@
     <xf numFmtId="164" fontId="18" fillId="7" borderId="26" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="16" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="16" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="16" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="18" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1869,16 +1868,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="16" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="18" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="2" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1902,14 +1892,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="2" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="7" borderId="2" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -2479,152 +2463,152 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F24"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="26" style="1" customWidth="1"/>
-    <col min="2" max="2" width="30.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="16.5703125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="22.7109375" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="1"/>
+    <col min="2" max="2" width="30.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="19.109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.88671875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="22.6640625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="37.5" customHeight="1">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
     </row>
     <row r="2" spans="1:6" ht="72" customHeight="1">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="44" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
     </row>
     <row r="3" spans="1:6" ht="31.5" customHeight="1">
-      <c r="A3" s="52"/>
-      <c r="B3" s="52"/>
-      <c r="C3" s="53" t="s">
+      <c r="A3" s="46"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="47" t="s">
         <v>72</v>
       </c>
-      <c r="D3" s="52"/>
-      <c r="E3" s="65" t="s">
+      <c r="D3" s="46"/>
+      <c r="E3" s="59" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="52"/>
+      <c r="F3" s="46"/>
     </row>
     <row r="4" spans="1:6" ht="29.25" customHeight="1">
-      <c r="A4" s="52"/>
-      <c r="B4" s="52"/>
-      <c r="C4" s="53" t="s">
+      <c r="A4" s="46"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53" t="s">
+      <c r="D4" s="46"/>
+      <c r="E4" s="47" t="s">
         <v>74</v>
       </c>
-      <c r="F4" s="52"/>
+      <c r="F4" s="46"/>
     </row>
     <row r="5" spans="1:6" ht="107.25" customHeight="1">
-      <c r="A5" s="65" t="s">
+      <c r="A5" s="59" t="s">
         <v>71</v>
       </c>
-      <c r="B5" s="53"/>
-      <c r="C5" s="49"/>
-      <c r="D5" s="49"/>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
+      <c r="B5" s="47"/>
+      <c r="C5" s="43"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
     </row>
     <row r="6" spans="1:6" ht="30" customHeight="1">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="5" t="s">
         <v>62</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="43" t="s">
+      <c r="C6" s="37" t="s">
         <v>70</v>
       </c>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="45"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="39"/>
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="5" t="s">
         <v>69</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C7" s="46"/>
-      <c r="D7" s="47"/>
-      <c r="E7" s="47"/>
-      <c r="F7" s="48"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="42"/>
     </row>
     <row r="8" spans="1:6" ht="22.5" customHeight="1">
-      <c r="A8" s="55" t="s">
+      <c r="A8" s="49" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="56"/>
-      <c r="C8" s="56"/>
-      <c r="D8" s="56"/>
-      <c r="E8" s="56"/>
-      <c r="F8" s="57"/>
-    </row>
-    <row r="9" spans="1:6" s="30" customFormat="1" ht="24.95" customHeight="1">
-      <c r="A9" s="41" t="s">
+      <c r="B8" s="50"/>
+      <c r="C8" s="50"/>
+      <c r="D8" s="50"/>
+      <c r="E8" s="50"/>
+      <c r="F8" s="51"/>
+    </row>
+    <row r="9" spans="1:6" s="22" customFormat="1" ht="24.9" customHeight="1">
+      <c r="A9" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="41" t="s">
+      <c r="B9" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="41" t="s">
+      <c r="C9" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="D9" s="41" t="s">
+      <c r="D9" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="41" t="s">
+      <c r="E9" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="F9" s="41" t="s">
+      <c r="F9" s="33" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="27.75" customHeight="1">
-      <c r="A10" s="28"/>
-      <c r="B10" s="31"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="33"/>
-    </row>
-    <row r="11" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A11" s="13"/>
+      <c r="A10" s="20"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+    </row>
+    <row r="11" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
     </row>
-    <row r="12" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A12" s="16"/>
+    <row r="12" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A12" s="4"/>
       <c r="B12" s="6"/>
       <c r="C12" s="4"/>
       <c r="D12" s="6"/>
       <c r="E12" s="7"/>
       <c r="F12" s="9"/>
     </row>
-    <row r="13" spans="1:6" ht="24.95" customHeight="1">
+    <row r="13" spans="1:6" ht="24.9" customHeight="1">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -2632,15 +2616,15 @@
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
     </row>
-    <row r="14" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A14" s="16"/>
+    <row r="14" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A14" s="4"/>
       <c r="B14" s="6"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
     </row>
-    <row r="15" spans="1:6" ht="24.95" customHeight="1">
+    <row r="15" spans="1:6" ht="24.9" customHeight="1">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -2648,7 +2632,7 @@
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
     </row>
-    <row r="16" spans="1:6" ht="24.95" customHeight="1">
+    <row r="16" spans="1:6" ht="24.9" customHeight="1">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -2656,7 +2640,7 @@
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
     </row>
-    <row r="17" spans="1:6" ht="24.95" customHeight="1">
+    <row r="17" spans="1:6" ht="24.9" customHeight="1">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -2664,7 +2648,7 @@
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
     </row>
-    <row r="18" spans="1:6" ht="24.95" customHeight="1">
+    <row r="18" spans="1:6" ht="24.9" customHeight="1">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -2672,75 +2656,70 @@
       <c r="E18" s="10"/>
       <c r="F18" s="10"/>
     </row>
-    <row r="19" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A19" s="35"/>
-      <c r="B19" s="35"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="36"/>
-      <c r="F19" s="36"/>
+    <row r="19" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A19" s="27"/>
+      <c r="B19" s="27"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
     </row>
     <row r="20" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A20" s="61" t="s">
+      <c r="A20" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="B20" s="62"/>
-      <c r="C20" s="62"/>
-      <c r="D20" s="62"/>
-      <c r="E20" s="63"/>
-      <c r="F20" s="34"/>
-    </row>
-    <row r="21" spans="1:6" ht="39.950000000000003" customHeight="1">
-      <c r="A21" s="50" t="s">
+      <c r="B20" s="56"/>
+      <c r="C20" s="56"/>
+      <c r="D20" s="56"/>
+      <c r="E20" s="57"/>
+      <c r="F20" s="26"/>
+    </row>
+    <row r="21" spans="1:6" ht="39.9" customHeight="1">
+      <c r="A21" s="44" t="s">
         <v>75</v>
       </c>
-      <c r="B21" s="50"/>
-      <c r="C21" s="64" t="s">
+      <c r="B21" s="44"/>
+      <c r="C21" s="58" t="s">
         <v>68</v>
       </c>
-      <c r="D21" s="51"/>
-      <c r="E21" s="51"/>
-      <c r="F21" s="23" t="s">
+      <c r="D21" s="45"/>
+      <c r="E21" s="45"/>
+      <c r="F21" s="16" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="39.950000000000003" customHeight="1">
-      <c r="A22" s="53"/>
-      <c r="B22" s="53"/>
-      <c r="C22" s="58" t="s">
+    <row r="22" spans="1:6" ht="39.9" customHeight="1">
+      <c r="A22" s="47"/>
+      <c r="B22" s="47"/>
+      <c r="C22" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="D22" s="59"/>
-      <c r="E22" s="59"/>
-      <c r="F22" s="60"/>
-    </row>
-    <row r="23" spans="1:6" ht="39.950000000000003" customHeight="1">
-      <c r="A23" s="53"/>
-      <c r="B23" s="53"/>
-      <c r="C23" s="53" t="s">
+      <c r="D22" s="53"/>
+      <c r="E22" s="53"/>
+      <c r="F22" s="54"/>
+    </row>
+    <row r="23" spans="1:6" ht="39.9" customHeight="1">
+      <c r="A23" s="47"/>
+      <c r="B23" s="47"/>
+      <c r="C23" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="D23" s="52"/>
-      <c r="E23" s="52"/>
-      <c r="F23" s="52"/>
+      <c r="D23" s="46"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
     </row>
     <row r="24" spans="1:6" ht="102.75" customHeight="1">
-      <c r="A24" s="53"/>
-      <c r="B24" s="53"/>
-      <c r="C24" s="53" t="s">
+      <c r="A24" s="47"/>
+      <c r="B24" s="47"/>
+      <c r="C24" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="D24" s="52"/>
-      <c r="E24" s="52"/>
-      <c r="F24" s="52"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="C6:F7"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="A2:B4"/>
-    <mergeCell ref="C24:F24"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="C22:F22"/>
@@ -2753,6 +2732,11 @@
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="C6:F7"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="A2:B4"/>
+    <mergeCell ref="C24:F24"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -2767,278 +2751,276 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F24"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="2" width="30.7109375" style="1" customWidth="1"/>
-    <col min="3" max="6" width="15.7109375" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="2" width="30.6640625" style="1" customWidth="1"/>
+    <col min="3" max="6" width="15.6640625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="35.25" customHeight="1">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
     </row>
     <row r="2" spans="1:6" ht="72" customHeight="1">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="44" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="89"/>
-      <c r="D2" s="89"/>
-      <c r="E2" s="89"/>
-      <c r="F2" s="89"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
     </row>
     <row r="3" spans="1:6" ht="30" customHeight="1">
-      <c r="A3" s="52"/>
-      <c r="B3" s="52"/>
-      <c r="C3" s="53" t="s">
+      <c r="A3" s="46"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="D3" s="52"/>
-      <c r="E3" s="90" t="s">
+      <c r="D3" s="46"/>
+      <c r="E3" s="61" t="s">
         <v>57</v>
       </c>
-      <c r="F3" s="52"/>
+      <c r="F3" s="46"/>
     </row>
     <row r="4" spans="1:6" ht="30" customHeight="1">
-      <c r="A4" s="52"/>
-      <c r="B4" s="52"/>
-      <c r="C4" s="53" t="s">
+      <c r="A4" s="46"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="47" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53"/>
-      <c r="F4" s="52"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="46"/>
     </row>
     <row r="5" spans="1:6" ht="112.5" customHeight="1">
-      <c r="A5" s="65" t="s">
+      <c r="A5" s="59" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="53"/>
-      <c r="C5" s="52" t="s">
+      <c r="B5" s="47"/>
+      <c r="C5" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
     </row>
     <row r="6" spans="1:6" ht="30" customHeight="1">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="65" t="s">
+      <c r="C6" s="59" t="s">
         <v>63</v>
       </c>
-      <c r="D6" s="65"/>
-      <c r="E6" s="53" t="s">
+      <c r="D6" s="59"/>
+      <c r="E6" s="47" t="s">
         <v>64</v>
       </c>
-      <c r="F6" s="53"/>
-    </row>
-    <row r="7" spans="1:6" ht="30">
-      <c r="A7" s="11" t="s">
+      <c r="F6" s="47"/>
+    </row>
+    <row r="7" spans="1:6" ht="28.8">
+      <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C7" s="52" t="s">
+      <c r="C7" s="46" t="s">
         <v>54</v>
       </c>
-      <c r="D7" s="52"/>
-      <c r="E7" s="79" t="s">
+      <c r="D7" s="46"/>
+      <c r="E7" s="67" t="s">
         <v>44</v>
       </c>
-      <c r="F7" s="79"/>
+      <c r="F7" s="67"/>
     </row>
     <row r="8" spans="1:6" ht="26.25" customHeight="1">
-      <c r="A8" s="74" t="s">
+      <c r="A8" s="62" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="75"/>
-      <c r="D8" s="75"/>
-      <c r="E8" s="75"/>
-      <c r="F8" s="76"/>
+      <c r="B8" s="63"/>
+      <c r="C8" s="63"/>
+      <c r="D8" s="63"/>
+      <c r="E8" s="63"/>
+      <c r="F8" s="64"/>
     </row>
     <row r="9" spans="1:6" ht="27" customHeight="1">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="21" t="s">
+      <c r="E9" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="F9" s="17" t="s">
+      <c r="F9" s="12" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="33" customHeight="1">
-      <c r="A10" s="16"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="16"/>
+      <c r="A10" s="4"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="4"/>
       <c r="D10" s="6"/>
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
     </row>
     <row r="11" spans="1:6" ht="21.75" customHeight="1">
-      <c r="A11" s="16"/>
-      <c r="B11" s="42"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
+      <c r="A11" s="4"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
     </row>
-    <row r="12" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A12" s="118"/>
-      <c r="B12" s="118"/>
-      <c r="C12" s="118"/>
-      <c r="D12" s="118"/>
-      <c r="E12" s="118"/>
-      <c r="F12" s="118"/>
-    </row>
-    <row r="13" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A13" s="118"/>
-      <c r="B13" s="118"/>
-      <c r="C13" s="118"/>
-      <c r="D13" s="118"/>
-      <c r="E13" s="118"/>
-      <c r="F13" s="118"/>
-    </row>
-    <row r="14" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A14" s="118"/>
-      <c r="B14" s="118"/>
-      <c r="C14" s="118"/>
-      <c r="D14" s="118"/>
-      <c r="E14" s="118"/>
-      <c r="F14" s="118"/>
-    </row>
-    <row r="15" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A15" s="118"/>
-      <c r="B15" s="118"/>
-      <c r="C15" s="118"/>
-      <c r="D15" s="118"/>
-      <c r="E15" s="118"/>
-      <c r="F15" s="118"/>
-    </row>
-    <row r="16" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A16" s="118"/>
-      <c r="B16" s="118"/>
-      <c r="C16" s="118"/>
-      <c r="D16" s="118"/>
-      <c r="E16" s="118"/>
-      <c r="F16" s="118"/>
-    </row>
-    <row r="17" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A17" s="118"/>
-      <c r="B17" s="118"/>
-      <c r="C17" s="118"/>
-      <c r="D17" s="118"/>
-      <c r="E17" s="118"/>
-      <c r="F17" s="118"/>
-    </row>
-    <row r="18" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A18" s="118"/>
-      <c r="B18" s="118"/>
-      <c r="C18" s="118"/>
-      <c r="D18" s="118"/>
-      <c r="E18" s="118"/>
-      <c r="F18" s="118"/>
+    <row r="12" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A12" s="35"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="35"/>
+    </row>
+    <row r="13" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A13" s="35"/>
+      <c r="B13" s="35"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="35"/>
+    </row>
+    <row r="14" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A14" s="35"/>
+      <c r="B14" s="35"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
+    </row>
+    <row r="15" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A15" s="35"/>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="35"/>
+    </row>
+    <row r="16" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A16" s="35"/>
+      <c r="B16" s="35"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="35"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="35"/>
+    </row>
+    <row r="17" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A17" s="35"/>
+      <c r="B17" s="35"/>
+      <c r="C17" s="35"/>
+      <c r="D17" s="35"/>
+      <c r="E17" s="35"/>
+      <c r="F17" s="35"/>
+    </row>
+    <row r="18" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A18" s="35"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="35"/>
+      <c r="F18" s="35"/>
     </row>
     <row r="19" spans="1:6" ht="20.25" customHeight="1">
-      <c r="A19" s="80" t="s">
+      <c r="A19" s="68" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="81"/>
-      <c r="C19" s="71" t="s">
+      <c r="B19" s="69"/>
+      <c r="C19" s="81" t="s">
         <v>17</v>
       </c>
-      <c r="D19" s="72"/>
-      <c r="E19" s="73"/>
-      <c r="F19" s="37"/>
+      <c r="D19" s="82"/>
+      <c r="E19" s="83"/>
+      <c r="F19" s="29"/>
     </row>
     <row r="20" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A20" s="82" t="s">
+      <c r="A20" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="83"/>
-      <c r="C20" s="83"/>
-      <c r="D20" s="83"/>
-      <c r="E20" s="83"/>
-      <c r="F20" s="84"/>
+      <c r="B20" s="71"/>
+      <c r="C20" s="71"/>
+      <c r="D20" s="71"/>
+      <c r="E20" s="71"/>
+      <c r="F20" s="72"/>
     </row>
     <row r="21" spans="1:6" ht="51.75" customHeight="1">
-      <c r="A21" s="69"/>
-      <c r="B21" s="70"/>
-      <c r="C21" s="77" t="s">
+      <c r="A21" s="79"/>
+      <c r="B21" s="80"/>
+      <c r="C21" s="65" t="s">
         <v>48</v>
       </c>
-      <c r="D21" s="78"/>
-      <c r="E21" s="78"/>
-      <c r="F21" s="11" t="s">
+      <c r="D21" s="66"/>
+      <c r="E21" s="66"/>
+      <c r="F21" s="5" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="30.75" customHeight="1">
-      <c r="A22" s="85" t="s">
+      <c r="A22" s="73" t="s">
         <v>66</v>
       </c>
-      <c r="B22" s="86"/>
-      <c r="C22" s="58" t="s">
+      <c r="B22" s="74"/>
+      <c r="C22" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="D22" s="59"/>
-      <c r="E22" s="59"/>
-      <c r="F22" s="60"/>
+      <c r="D22" s="53"/>
+      <c r="E22" s="53"/>
+      <c r="F22" s="54"/>
     </row>
     <row r="23" spans="1:6" ht="30.75" customHeight="1">
-      <c r="A23" s="87"/>
-      <c r="B23" s="88"/>
-      <c r="C23" s="53" t="s">
+      <c r="A23" s="75"/>
+      <c r="B23" s="76"/>
+      <c r="C23" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="D23" s="52"/>
-      <c r="E23" s="52"/>
-      <c r="F23" s="52"/>
+      <c r="D23" s="46"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
     </row>
     <row r="24" spans="1:6" ht="86.25" customHeight="1">
-      <c r="A24" s="67" t="s">
+      <c r="A24" s="77" t="s">
         <v>42</v>
       </c>
-      <c r="B24" s="68"/>
-      <c r="C24" s="53" t="s">
+      <c r="B24" s="78"/>
+      <c r="C24" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="D24" s="52"/>
-      <c r="E24" s="52"/>
-      <c r="F24" s="52"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:B4"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="C24:F24"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:F5"/>
     <mergeCell ref="A8:F8"/>
@@ -3051,11 +3033,13 @@
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A20:F20"/>
     <mergeCell ref="A22:B23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C23:F23"/>
-    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:B4"/>
+    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
   </mergeCells>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="79" orientation="portrait" horizontalDpi="300" r:id="rId1"/>
@@ -3069,138 +3053,138 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F24"/>
-  <sheetFormatPr defaultRowHeight="46.5" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="46.5" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="30.7109375" style="1" customWidth="1"/>
-    <col min="3" max="6" width="15.7109375" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="2" width="30.6640625" style="1" customWidth="1"/>
+    <col min="3" max="6" width="15.6640625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36.75" customHeight="1">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="48" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
     </row>
     <row r="2" spans="1:6" ht="60" customHeight="1">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="108"/>
-      <c r="D2" s="108"/>
-      <c r="E2" s="108"/>
-      <c r="F2" s="108"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
     </row>
     <row r="3" spans="1:6" ht="30" customHeight="1">
-      <c r="A3" s="52"/>
-      <c r="B3" s="52"/>
-      <c r="C3" s="53" t="s">
+      <c r="A3" s="46"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="D3" s="52"/>
-      <c r="E3" s="65" t="s">
+      <c r="D3" s="46"/>
+      <c r="E3" s="59" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="52"/>
+      <c r="F3" s="46"/>
     </row>
     <row r="4" spans="1:6" ht="30" customHeight="1">
-      <c r="A4" s="52"/>
-      <c r="B4" s="52"/>
-      <c r="C4" s="53" t="s">
+      <c r="A4" s="46"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53" t="s">
+      <c r="D4" s="46"/>
+      <c r="E4" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="F4" s="52"/>
+      <c r="F4" s="46"/>
     </row>
     <row r="5" spans="1:6" ht="120" customHeight="1">
-      <c r="A5" s="65" t="s">
+      <c r="A5" s="59" t="s">
         <v>76</v>
       </c>
-      <c r="B5" s="53"/>
-      <c r="C5" s="52" t="s">
+      <c r="B5" s="47"/>
+      <c r="C5" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
     </row>
     <row r="6" spans="1:6" ht="30" customHeight="1">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="65" t="s">
+      <c r="C6" s="59" t="s">
         <v>77</v>
       </c>
-      <c r="D6" s="65"/>
-      <c r="E6" s="53" t="s">
+      <c r="D6" s="59"/>
+      <c r="E6" s="47" t="s">
         <v>78</v>
       </c>
-      <c r="F6" s="53"/>
+      <c r="F6" s="47"/>
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C7" s="52" t="s">
+      <c r="C7" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="52"/>
-      <c r="E7" s="107"/>
-      <c r="F7" s="107"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="86"/>
+      <c r="F7" s="86"/>
     </row>
     <row r="8" spans="1:6" ht="27" customHeight="1">
-      <c r="A8" s="74" t="s">
+      <c r="A8" s="62" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="75"/>
-      <c r="D8" s="75"/>
-      <c r="E8" s="75"/>
-      <c r="F8" s="76"/>
-    </row>
-    <row r="9" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A9" s="17" t="s">
+      <c r="B8" s="63"/>
+      <c r="C8" s="63"/>
+      <c r="D8" s="63"/>
+      <c r="E8" s="63"/>
+      <c r="F8" s="64"/>
+    </row>
+    <row r="9" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A9" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="17" t="s">
+      <c r="E9" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="17" t="s">
+      <c r="F9" s="12" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="30.75" customHeight="1">
       <c r="A10" s="4"/>
-      <c r="B10" s="12"/>
+      <c r="B10" s="11"/>
       <c r="C10" s="4"/>
       <c r="D10" s="6"/>
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
     </row>
-    <row r="11" spans="1:6" ht="24.95" customHeight="1">
+    <row r="11" spans="1:6" ht="24.9" customHeight="1">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -3208,7 +3192,7 @@
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
     </row>
-    <row r="12" spans="1:6" ht="24.95" customHeight="1">
+    <row r="12" spans="1:6" ht="24.9" customHeight="1">
       <c r="A12" s="4"/>
       <c r="B12" s="6"/>
       <c r="C12" s="4"/>
@@ -3216,7 +3200,7 @@
       <c r="E12" s="7"/>
       <c r="F12" s="9"/>
     </row>
-    <row r="13" spans="1:6" ht="24.95" customHeight="1">
+    <row r="13" spans="1:6" ht="24.9" customHeight="1">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -3224,135 +3208,118 @@
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
     </row>
-    <row r="14" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A14" s="93" t="s">
+    <row r="14" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A14" s="89" t="s">
         <v>79</v>
       </c>
-      <c r="B14" s="94"/>
+      <c r="B14" s="90"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
     </row>
-    <row r="15" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A15" s="95"/>
-      <c r="B15" s="96"/>
+    <row r="15" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A15" s="91"/>
+      <c r="B15" s="92"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
       <c r="E15" s="7"/>
       <c r="F15" s="7"/>
     </row>
-    <row r="16" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A16" s="95"/>
-      <c r="B16" s="96"/>
+    <row r="16" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A16" s="91"/>
+      <c r="B16" s="92"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
       <c r="E16" s="7"/>
       <c r="F16" s="7"/>
     </row>
-    <row r="17" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A17" s="95"/>
-      <c r="B17" s="96"/>
+    <row r="17" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A17" s="91"/>
+      <c r="B17" s="92"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
     </row>
-    <row r="18" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A18" s="97"/>
-      <c r="B18" s="98"/>
+    <row r="18" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A18" s="93"/>
+      <c r="B18" s="94"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
       <c r="E18" s="7"/>
       <c r="F18" s="7"/>
     </row>
     <row r="19" spans="1:6" ht="21" customHeight="1">
-      <c r="A19" s="80" t="s">
+      <c r="A19" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="81"/>
-      <c r="C19" s="72" t="s">
+      <c r="B19" s="69"/>
+      <c r="C19" s="82" t="s">
         <v>17</v>
       </c>
-      <c r="D19" s="72"/>
-      <c r="E19" s="72"/>
-      <c r="F19" s="37"/>
+      <c r="D19" s="82"/>
+      <c r="E19" s="82"/>
+      <c r="F19" s="29"/>
     </row>
     <row r="20" spans="1:6" ht="47.25" hidden="1" customHeight="1">
-      <c r="A20" s="82" t="s">
+      <c r="A20" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="83"/>
-      <c r="C20" s="83"/>
-      <c r="D20" s="83"/>
-      <c r="E20" s="83"/>
-      <c r="F20" s="84"/>
+      <c r="B20" s="71"/>
+      <c r="C20" s="71"/>
+      <c r="D20" s="71"/>
+      <c r="E20" s="71"/>
+      <c r="F20" s="72"/>
     </row>
     <row r="21" spans="1:6" ht="72" customHeight="1">
-      <c r="A21" s="99" t="s">
+      <c r="A21" s="95" t="s">
         <v>86</v>
       </c>
-      <c r="B21" s="100"/>
-      <c r="C21" s="105" t="s">
+      <c r="B21" s="96"/>
+      <c r="C21" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="D21" s="106"/>
-      <c r="E21" s="106"/>
-      <c r="F21" s="11" t="s">
+      <c r="D21" s="85"/>
+      <c r="E21" s="85"/>
+      <c r="F21" s="5" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="30" customHeight="1">
-      <c r="A22" s="101"/>
-      <c r="B22" s="102"/>
-      <c r="C22" s="58" t="s">
+      <c r="A22" s="97"/>
+      <c r="B22" s="98"/>
+      <c r="C22" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="D22" s="59"/>
-      <c r="E22" s="59"/>
-      <c r="F22" s="60"/>
+      <c r="D22" s="53"/>
+      <c r="E22" s="53"/>
+      <c r="F22" s="54"/>
     </row>
     <row r="23" spans="1:6" ht="30" customHeight="1">
-      <c r="A23" s="103"/>
-      <c r="B23" s="104"/>
-      <c r="C23" s="53" t="s">
+      <c r="A23" s="99"/>
+      <c r="B23" s="100"/>
+      <c r="C23" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="D23" s="52"/>
-      <c r="E23" s="52"/>
-      <c r="F23" s="52"/>
+      <c r="D23" s="46"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
     </row>
     <row r="24" spans="1:6" ht="66.75" customHeight="1">
-      <c r="A24" s="91" t="s">
+      <c r="A24" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="92"/>
-      <c r="C24" s="53" t="s">
+      <c r="B24" s="88"/>
+      <c r="C24" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="D24" s="52"/>
-      <c r="E24" s="52"/>
-      <c r="F24" s="52"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:B4"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:F7"/>
     <mergeCell ref="C22:F22"/>
     <mergeCell ref="C23:F23"/>
     <mergeCell ref="A24:B24"/>
@@ -3360,595 +3327,10 @@
     <mergeCell ref="A14:B18"/>
     <mergeCell ref="A21:B23"/>
     <mergeCell ref="C19:E19"/>
-  </mergeCells>
-  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="256" scale="81" orientation="portrait" horizontalDpi="300" r:id="rId1"/>
-  <drawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7E100D8-CE6E-40F1-8413-A338847C2C66}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:F23"/>
-  <sheetFormatPr defaultRowHeight="46.5" customHeight="1"/>
-  <cols>
-    <col min="1" max="2" width="30.7109375" style="1" customWidth="1"/>
-    <col min="3" max="6" width="15.7109375" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" ht="34.5" customHeight="1">
-      <c r="A1" s="116" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" s="116"/>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-    </row>
-    <row r="2" spans="1:6" ht="60" customHeight="1">
-      <c r="A2" s="50" t="s">
-        <v>53</v>
-      </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="89"/>
-      <c r="D2" s="89"/>
-      <c r="E2" s="89"/>
-      <c r="F2" s="89"/>
-    </row>
-    <row r="3" spans="1:6" ht="30" customHeight="1">
-      <c r="A3" s="52"/>
-      <c r="B3" s="52"/>
-      <c r="C3" s="58" t="s">
-        <v>81</v>
-      </c>
-      <c r="D3" s="60"/>
-      <c r="E3" s="65" t="s">
-        <v>73</v>
-      </c>
-      <c r="F3" s="52"/>
-    </row>
-    <row r="4" spans="1:6" ht="30" customHeight="1">
-      <c r="A4" s="52"/>
-      <c r="B4" s="52"/>
-      <c r="C4" s="53" t="s">
-        <v>58</v>
-      </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53" t="s">
-        <v>49</v>
-      </c>
-      <c r="F4" s="52"/>
-    </row>
-    <row r="5" spans="1:6" ht="124.5" customHeight="1">
-      <c r="A5" s="65" t="s">
-        <v>80</v>
-      </c>
-      <c r="B5" s="53"/>
-      <c r="C5" s="52" t="s">
-        <v>39</v>
-      </c>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-    </row>
-    <row r="6" spans="1:6" ht="30" customHeight="1">
-      <c r="A6" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" s="65" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="65"/>
-      <c r="E6" s="53" t="s">
-        <v>83</v>
-      </c>
-      <c r="F6" s="53"/>
-    </row>
-    <row r="7" spans="1:6" ht="30" customHeight="1">
-      <c r="A7" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="52" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="52"/>
-      <c r="E7" s="107"/>
-      <c r="F7" s="107"/>
-    </row>
-    <row r="8" spans="1:6" ht="27" customHeight="1">
-      <c r="A8" s="74" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="75"/>
-      <c r="D8" s="75"/>
-      <c r="E8" s="75"/>
-      <c r="F8" s="76"/>
-    </row>
-    <row r="9" spans="1:6" ht="30.75" customHeight="1">
-      <c r="A9" s="17" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>45</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="17" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="21" customHeight="1">
-      <c r="A10" s="16"/>
-      <c r="B10" s="42"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-    </row>
-    <row r="11" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A11" s="4"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="20"/>
-    </row>
-    <row r="12" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A12" s="26"/>
-      <c r="B12" s="26"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-    </row>
-    <row r="13" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A13" s="27" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="27"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-    </row>
-    <row r="14" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A14" s="27"/>
-      <c r="B14" s="27"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-    </row>
-    <row r="15" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A15" s="27"/>
-      <c r="B15" s="27"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-    </row>
-    <row r="16" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A16" s="27"/>
-      <c r="B16" s="27"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-    </row>
-    <row r="17" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A17" s="29"/>
-      <c r="B17" s="29"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-    </row>
-    <row r="18" spans="1:6" ht="21" customHeight="1">
-      <c r="A18" s="71" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18" s="73"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="38">
-        <f>SUM(E10:E17)</f>
-        <v>0</v>
-      </c>
-      <c r="F18" s="40">
-        <f>SUM(F10:F17)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="47.25" hidden="1" customHeight="1">
-      <c r="A19" s="82" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19" s="83"/>
-      <c r="C19" s="83"/>
-      <c r="D19" s="83"/>
-      <c r="E19" s="83"/>
-      <c r="F19" s="84"/>
-    </row>
-    <row r="20" spans="1:6" ht="72" customHeight="1">
-      <c r="A20" s="85" t="s">
-        <v>82</v>
-      </c>
-      <c r="B20" s="86"/>
-      <c r="C20" s="111" t="s">
-        <v>46</v>
-      </c>
-      <c r="D20" s="112"/>
-      <c r="E20" s="112"/>
-      <c r="F20" s="113"/>
-    </row>
-    <row r="21" spans="1:6" ht="30" customHeight="1">
-      <c r="A21" s="114"/>
-      <c r="B21" s="115"/>
-      <c r="C21" s="58" t="s">
-        <v>9</v>
-      </c>
-      <c r="D21" s="59"/>
-      <c r="E21" s="59"/>
-      <c r="F21" s="60"/>
-    </row>
-    <row r="22" spans="1:6" ht="30" customHeight="1">
-      <c r="A22" s="87"/>
-      <c r="B22" s="88"/>
-      <c r="C22" s="53" t="s">
-        <v>10</v>
-      </c>
-      <c r="D22" s="52"/>
-      <c r="E22" s="52"/>
-      <c r="F22" s="52"/>
-    </row>
-    <row r="23" spans="1:6" ht="66.75" customHeight="1">
-      <c r="A23" s="109" t="s">
-        <v>47</v>
-      </c>
-      <c r="B23" s="110"/>
-      <c r="C23" s="53" t="s">
-        <v>11</v>
-      </c>
-      <c r="D23" s="52"/>
-      <c r="E23" s="52"/>
-      <c r="F23" s="52"/>
-    </row>
-  </sheetData>
-  <mergeCells count="22">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:B4"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="C23:F23"/>
-    <mergeCell ref="C20:F20"/>
     <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A20:B22"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="C22:F22"/>
-  </mergeCells>
-  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="79" orientation="portrait" horizontalDpi="300" r:id="rId1"/>
-  <drawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36F50A3D-8B8D-48D1-9B30-CA99D8C88528}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:F24"/>
-  <sheetFormatPr defaultRowHeight="46.5" customHeight="1"/>
-  <cols>
-    <col min="1" max="2" width="30.7109375" style="1" customWidth="1"/>
-    <col min="3" max="6" width="15.7109375" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" ht="32.25" customHeight="1">
-      <c r="A1" s="117" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-    </row>
-    <row r="2" spans="1:6" ht="60" customHeight="1">
-      <c r="A2" s="50" t="s">
-        <v>53</v>
-      </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="89"/>
-      <c r="D2" s="89"/>
-      <c r="E2" s="89"/>
-      <c r="F2" s="89"/>
-    </row>
-    <row r="3" spans="1:6" ht="30" customHeight="1">
-      <c r="A3" s="52"/>
-      <c r="B3" s="52"/>
-      <c r="C3" s="53" t="s">
-        <v>58</v>
-      </c>
-      <c r="D3" s="52"/>
-      <c r="E3" s="65" t="s">
-        <v>73</v>
-      </c>
-      <c r="F3" s="52"/>
-    </row>
-    <row r="4" spans="1:6" ht="30" customHeight="1">
-      <c r="A4" s="52"/>
-      <c r="B4" s="52"/>
-      <c r="C4" s="53" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="53" t="s">
-        <v>52</v>
-      </c>
-      <c r="F4" s="52"/>
-    </row>
-    <row r="5" spans="1:6" ht="120" customHeight="1">
-      <c r="A5" s="65" t="s">
-        <v>84</v>
-      </c>
-      <c r="B5" s="53"/>
-      <c r="C5" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-    </row>
-    <row r="6" spans="1:6" ht="30" customHeight="1">
-      <c r="A6" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C6" s="65" t="s">
-        <v>77</v>
-      </c>
-      <c r="D6" s="65"/>
-      <c r="E6" s="53" t="s">
-        <v>78</v>
-      </c>
-      <c r="F6" s="53"/>
-    </row>
-    <row r="7" spans="1:6" ht="30" customHeight="1">
-      <c r="A7" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C7" s="52" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="52"/>
-      <c r="E7" s="52" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" s="52"/>
-    </row>
-    <row r="8" spans="1:6" ht="27" customHeight="1">
-      <c r="A8" s="74" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="75"/>
-      <c r="D8" s="75"/>
-      <c r="E8" s="75"/>
-      <c r="F8" s="76"/>
-    </row>
-    <row r="9" spans="1:6" ht="30.75" customHeight="1">
-      <c r="A9" s="17" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="17" t="s">
-        <v>4</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="F9" s="17" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="27.75" customHeight="1">
-      <c r="A10" s="16"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-    </row>
-    <row r="11" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A11" s="16"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-    </row>
-    <row r="12" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A12" s="16"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="9"/>
-    </row>
-    <row r="13" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A13" s="16"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-    </row>
-    <row r="14" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A14" s="93" t="s">
-        <v>31</v>
-      </c>
-      <c r="B14" s="94"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-    </row>
-    <row r="15" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A15" s="95"/>
-      <c r="B15" s="96"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-    </row>
-    <row r="16" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A16" s="95"/>
-      <c r="B16" s="96"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-    </row>
-    <row r="17" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A17" s="95"/>
-      <c r="B17" s="96"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-    </row>
-    <row r="18" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A18" s="97"/>
-      <c r="B18" s="98"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-    </row>
-    <row r="19" spans="1:6" ht="21" customHeight="1">
-      <c r="A19" s="80" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19" s="81"/>
-      <c r="C19" s="72" t="s">
-        <v>17</v>
-      </c>
-      <c r="D19" s="72"/>
-      <c r="E19" s="72"/>
-      <c r="F19" s="37"/>
-    </row>
-    <row r="20" spans="1:6" ht="47.25" hidden="1" customHeight="1">
-      <c r="A20" s="82" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20" s="83"/>
-      <c r="C20" s="83"/>
-      <c r="D20" s="83"/>
-      <c r="E20" s="83"/>
-      <c r="F20" s="84"/>
-    </row>
-    <row r="21" spans="1:6" ht="72" customHeight="1">
-      <c r="A21" s="53" t="s">
-        <v>85</v>
-      </c>
-      <c r="B21" s="53"/>
-      <c r="C21" s="105" t="s">
-        <v>24</v>
-      </c>
-      <c r="D21" s="106"/>
-      <c r="E21" s="106"/>
-      <c r="F21" s="14" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="30" customHeight="1">
-      <c r="A22" s="53"/>
-      <c r="B22" s="53"/>
-      <c r="C22" s="58" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" s="59"/>
-      <c r="E22" s="59"/>
-      <c r="F22" s="60"/>
-    </row>
-    <row r="23" spans="1:6" ht="30" customHeight="1">
-      <c r="A23" s="53"/>
-      <c r="B23" s="53"/>
-      <c r="C23" s="53" t="s">
-        <v>10</v>
-      </c>
-      <c r="D23" s="52"/>
-      <c r="E23" s="52"/>
-      <c r="F23" s="52"/>
-    </row>
-    <row r="24" spans="1:6" ht="66.75" customHeight="1">
-      <c r="A24" s="91" t="s">
-        <v>25</v>
-      </c>
-      <c r="B24" s="92"/>
-      <c r="C24" s="53" t="s">
-        <v>11</v>
-      </c>
-      <c r="D24" s="52"/>
-      <c r="E24" s="52"/>
-      <c r="F24" s="52"/>
-    </row>
-  </sheetData>
-  <mergeCells count="24">
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:F24"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A14:B18"/>
     <mergeCell ref="A19:B19"/>
-    <mergeCell ref="C19:E19"/>
     <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A21:B23"/>
     <mergeCell ref="C21:E21"/>
-    <mergeCell ref="C22:F22"/>
-    <mergeCell ref="C23:F23"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:F5"/>
     <mergeCell ref="C6:D6"/>
@@ -3964,6 +3346,608 @@
     <mergeCell ref="E4:F4"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="256" scale="81" orientation="portrait" horizontalDpi="300" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7E100D8-CE6E-40F1-8413-A338847C2C66}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="46.5" customHeight="1"/>
+  <cols>
+    <col min="1" max="2" width="30.6640625" style="1" customWidth="1"/>
+    <col min="3" max="6" width="15.6640625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="34.5" customHeight="1">
+      <c r="A1" s="101" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="101"/>
+      <c r="C1" s="101"/>
+      <c r="D1" s="101"/>
+      <c r="E1" s="101"/>
+      <c r="F1" s="101"/>
+    </row>
+    <row r="2" spans="1:6" ht="60" customHeight="1">
+      <c r="A2" s="44" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+    </row>
+    <row r="3" spans="1:6" ht="30" customHeight="1">
+      <c r="A3" s="46"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="52" t="s">
+        <v>81</v>
+      </c>
+      <c r="D3" s="54"/>
+      <c r="E3" s="59" t="s">
+        <v>73</v>
+      </c>
+      <c r="F3" s="46"/>
+    </row>
+    <row r="4" spans="1:6" ht="30" customHeight="1">
+      <c r="A4" s="46"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="47" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="46"/>
+      <c r="E4" s="47" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" s="46"/>
+    </row>
+    <row r="5" spans="1:6" ht="124.5" customHeight="1">
+      <c r="A5" s="59" t="s">
+        <v>80</v>
+      </c>
+      <c r="B5" s="47"/>
+      <c r="C5" s="46" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+    </row>
+    <row r="6" spans="1:6" ht="30" customHeight="1">
+      <c r="A6" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="59" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="59"/>
+      <c r="E6" s="47" t="s">
+        <v>83</v>
+      </c>
+      <c r="F6" s="47"/>
+    </row>
+    <row r="7" spans="1:6" ht="30" customHeight="1">
+      <c r="A7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="46"/>
+      <c r="E7" s="86"/>
+      <c r="F7" s="86"/>
+    </row>
+    <row r="8" spans="1:6" ht="27" customHeight="1">
+      <c r="A8" s="62" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="63"/>
+      <c r="C8" s="63"/>
+      <c r="D8" s="63"/>
+      <c r="E8" s="63"/>
+      <c r="F8" s="64"/>
+    </row>
+    <row r="9" spans="1:6" ht="30.75" customHeight="1">
+      <c r="A9" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="21" customHeight="1">
+      <c r="A10" s="4"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+    </row>
+    <row r="11" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A11" s="4"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="13"/>
+    </row>
+    <row r="12" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A12" s="15"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+    </row>
+    <row r="13" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A13" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="19"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+    </row>
+    <row r="14" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A14" s="19"/>
+      <c r="B14" s="19"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+    </row>
+    <row r="15" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A15" s="19"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+    </row>
+    <row r="16" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A16" s="19"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+    </row>
+    <row r="17" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A17" s="21"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+    </row>
+    <row r="18" spans="1:6" ht="21" customHeight="1">
+      <c r="A18" s="81" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="83"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="30">
+        <f>SUM(E10:E17)</f>
+        <v>0</v>
+      </c>
+      <c r="F18" s="32">
+        <f>SUM(F10:F17)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="47.25" hidden="1" customHeight="1">
+      <c r="A19" s="70" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="71"/>
+      <c r="C19" s="71"/>
+      <c r="D19" s="71"/>
+      <c r="E19" s="71"/>
+      <c r="F19" s="72"/>
+    </row>
+    <row r="20" spans="1:6" ht="72" customHeight="1">
+      <c r="A20" s="73" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" s="74"/>
+      <c r="C20" s="104" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="105"/>
+      <c r="E20" s="105"/>
+      <c r="F20" s="106"/>
+    </row>
+    <row r="21" spans="1:6" ht="30" customHeight="1">
+      <c r="A21" s="107"/>
+      <c r="B21" s="108"/>
+      <c r="C21" s="52" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" s="53"/>
+      <c r="E21" s="53"/>
+      <c r="F21" s="54"/>
+    </row>
+    <row r="22" spans="1:6" ht="30" customHeight="1">
+      <c r="A22" s="75"/>
+      <c r="B22" s="76"/>
+      <c r="C22" s="47" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="46"/>
+      <c r="E22" s="46"/>
+      <c r="F22" s="46"/>
+    </row>
+    <row r="23" spans="1:6" ht="66.75" customHeight="1">
+      <c r="A23" s="102" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" s="103"/>
+      <c r="C23" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="46"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
+    </row>
+  </sheetData>
+  <mergeCells count="22">
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A20:B22"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="C22:F22"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:B4"/>
+    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="C3:D3"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="79" orientation="portrait" horizontalDpi="300" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36F50A3D-8B8D-48D1-9B30-CA99D8C88528}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="46.5" customHeight="1"/>
+  <cols>
+    <col min="1" max="2" width="30.6640625" style="1" customWidth="1"/>
+    <col min="3" max="6" width="15.6640625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="32.25" customHeight="1">
+      <c r="A1" s="109" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="109"/>
+      <c r="C1" s="109"/>
+      <c r="D1" s="109"/>
+      <c r="E1" s="109"/>
+      <c r="F1" s="109"/>
+    </row>
+    <row r="2" spans="1:6" ht="60" customHeight="1">
+      <c r="A2" s="44" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+    </row>
+    <row r="3" spans="1:6" ht="30" customHeight="1">
+      <c r="A3" s="46"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="47" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="46"/>
+      <c r="E3" s="59" t="s">
+        <v>73</v>
+      </c>
+      <c r="F3" s="46"/>
+    </row>
+    <row r="4" spans="1:6" ht="30" customHeight="1">
+      <c r="A4" s="46"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="46"/>
+      <c r="E4" s="47" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="46"/>
+    </row>
+    <row r="5" spans="1:6" ht="120" customHeight="1">
+      <c r="A5" s="59" t="s">
+        <v>84</v>
+      </c>
+      <c r="B5" s="47"/>
+      <c r="C5" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+    </row>
+    <row r="6" spans="1:6" ht="30" customHeight="1">
+      <c r="A6" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="59" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" s="59"/>
+      <c r="E6" s="47" t="s">
+        <v>78</v>
+      </c>
+      <c r="F6" s="47"/>
+    </row>
+    <row r="7" spans="1:6" ht="30" customHeight="1">
+      <c r="A7" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="46"/>
+    </row>
+    <row r="8" spans="1:6" ht="27" customHeight="1">
+      <c r="A8" s="62" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="63"/>
+      <c r="C8" s="63"/>
+      <c r="D8" s="63"/>
+      <c r="E8" s="63"/>
+      <c r="F8" s="64"/>
+    </row>
+    <row r="9" spans="1:6" ht="30.75" customHeight="1">
+      <c r="A9" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="27.75" customHeight="1">
+      <c r="A10" s="4"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+    </row>
+    <row r="11" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+    </row>
+    <row r="12" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A12" s="4"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="9"/>
+    </row>
+    <row r="13" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+    </row>
+    <row r="14" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A14" s="89" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="90"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+    </row>
+    <row r="15" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A15" s="91"/>
+      <c r="B15" s="92"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+    </row>
+    <row r="16" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A16" s="91"/>
+      <c r="B16" s="92"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+    </row>
+    <row r="17" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A17" s="91"/>
+      <c r="B17" s="92"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+    </row>
+    <row r="18" spans="1:6" ht="24.9" customHeight="1">
+      <c r="A18" s="93"/>
+      <c r="B18" s="94"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+    </row>
+    <row r="19" spans="1:6" ht="21" customHeight="1">
+      <c r="A19" s="68" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="69"/>
+      <c r="C19" s="82" t="s">
+        <v>17</v>
+      </c>
+      <c r="D19" s="82"/>
+      <c r="E19" s="82"/>
+      <c r="F19" s="29"/>
+    </row>
+    <row r="20" spans="1:6" ht="47.25" hidden="1" customHeight="1">
+      <c r="A20" s="70" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="71"/>
+      <c r="C20" s="71"/>
+      <c r="D20" s="71"/>
+      <c r="E20" s="71"/>
+      <c r="F20" s="72"/>
+    </row>
+    <row r="21" spans="1:6" ht="72" customHeight="1">
+      <c r="A21" s="47" t="s">
+        <v>85</v>
+      </c>
+      <c r="B21" s="47"/>
+      <c r="C21" s="84" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" s="85"/>
+      <c r="E21" s="85"/>
+      <c r="F21" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="30" customHeight="1">
+      <c r="A22" s="47"/>
+      <c r="B22" s="47"/>
+      <c r="C22" s="52" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="53"/>
+      <c r="E22" s="53"/>
+      <c r="F22" s="54"/>
+    </row>
+    <row r="23" spans="1:6" ht="30" customHeight="1">
+      <c r="A23" s="47"/>
+      <c r="B23" s="47"/>
+      <c r="C23" s="47" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="46"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
+    </row>
+    <row r="24" spans="1:6" ht="66.75" customHeight="1">
+      <c r="A24" s="87" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" s="88"/>
+      <c r="C24" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="46"/>
+    </row>
+  </sheetData>
+  <mergeCells count="24">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:B4"/>
+    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A14:B18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A21:B23"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C22:F22"/>
+    <mergeCell ref="C23:F23"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="79" orientation="portrait" horizontalDpi="300" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>